<commit_message>
Refresh stock closing prices
</commit_message>
<xml_diff>
--- a/outputs/stock_closing_prices.xlsx
+++ b/outputs/stock_closing_prices.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closing Prices" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Closing Prices" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -449,92 +437,92 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Sector</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Company Name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>2026-04-29 Close</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>2026-04-29 Change</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>2026-04-29 Change %</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>2026-04-30 Close</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>2026-04-30 Change</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>2026-04-30 Change %</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>2026-05-04 Close</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>2026-05-04 Change</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>2026-05-04 Change %</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>2026-05-05 Close</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>2026-05-05 Change</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>2026-05-05 Change %</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>2026-05-06 Close</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>2026-05-06 Change</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>2026-05-06 Change %</t>
         </is>

</xml_diff>

<commit_message>
Align percent changes with displayed prices
</commit_message>
<xml_diff>
--- a/outputs/stock_closing_prices.xlsx
+++ b/outputs/stock_closing_prices.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Closing Prices" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closing Prices" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -437,92 +449,92 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Sector</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Company Name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>2026-04-29 Close</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>2026-04-29 Change</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>2026-04-29 Change %</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>2026-04-30 Close</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>2026-04-30 Change</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>2026-04-30 Change %</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>2026-05-04 Close</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>2026-05-04 Change</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>2026-05-04 Change %</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>2026-05-05 Close</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>2026-05-05 Change</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>2026-05-05 Change %</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>2026-05-06 Close</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>2026-05-06 Change</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>2026-05-06 Change %</t>
         </is>
@@ -2567,7 +2579,7 @@
         <v>0.08</v>
       </c>
       <c r="F35" t="n">
-        <v>1.78</v>
+        <v>1.69</v>
       </c>
       <c r="G35" t="n">
         <v>4.78</v>
@@ -2576,34 +2588,34 @@
         <v>-0.03</v>
       </c>
       <c r="I35" t="n">
-        <v>-0.71</v>
+        <v>-0.62</v>
       </c>
       <c r="J35" t="n">
         <v>4.87</v>
       </c>
       <c r="K35" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="L35" t="n">
-        <v>2.05</v>
+        <v>1.88</v>
       </c>
       <c r="M35" t="n">
         <v>4.82</v>
       </c>
       <c r="N35" t="n">
-        <v>-0.06</v>
+        <v>-0.05</v>
       </c>
       <c r="O35" t="n">
-        <v>-1.15</v>
+        <v>-1.03</v>
       </c>
       <c r="P35" t="n">
         <v>4.82</v>
       </c>
       <c r="Q35" t="n">
-        <v>-0.06</v>
+        <v>-0.05</v>
       </c>
       <c r="R35" t="n">
-        <v>-1.15</v>
+        <v>-1.03</v>
       </c>
     </row>
     <row r="36">
@@ -3367,7 +3379,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.35</v>
+        <v>0.355</v>
       </c>
       <c r="E48" t="n">
         <v>0</v>
@@ -3376,7 +3388,7 @@
         <v>0</v>
       </c>
       <c r="G48" t="n">
-        <v>0.34</v>
+        <v>0.345</v>
       </c>
       <c r="H48" t="n">
         <v>-0.01</v>
@@ -3385,7 +3397,7 @@
         <v>-2.82</v>
       </c>
       <c r="J48" t="n">
-        <v>0.35</v>
+        <v>0.355</v>
       </c>
       <c r="K48" t="n">
         <v>0.01</v>
@@ -3394,7 +3406,7 @@
         <v>2.9</v>
       </c>
       <c r="M48" t="n">
-        <v>0.38</v>
+        <v>0.375</v>
       </c>
       <c r="N48" t="n">
         <v>0.02</v>
@@ -3406,7 +3418,7 @@
         <v>0.38</v>
       </c>
       <c r="Q48" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="R48" t="n">
         <v>1.33</v>
@@ -3766,16 +3778,16 @@
         <v>2.38</v>
       </c>
       <c r="M54" t="n">
-        <v>0.43</v>
+        <v>0.425</v>
       </c>
       <c r="N54" t="n">
-        <v>-0</v>
+        <v>-0.005</v>
       </c>
       <c r="O54" t="n">
         <v>-1.16</v>
       </c>
       <c r="P54" t="n">
-        <v>0.43</v>
+        <v>0.425</v>
       </c>
       <c r="Q54" t="n">
         <v>0</v>
@@ -3801,10 +3813,10 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.7</v>
+        <v>0.705</v>
       </c>
       <c r="E55" t="n">
-        <v>-0</v>
+        <v>-0.005</v>
       </c>
       <c r="F55" t="n">
         <v>-0.7</v>
@@ -3813,7 +3825,7 @@
         <v>0.68</v>
       </c>
       <c r="H55" t="n">
-        <v>-0.02</v>
+        <v>-0.025</v>
       </c>
       <c r="I55" t="n">
         <v>-3.55</v>
@@ -3828,16 +3840,16 @@
         <v>0</v>
       </c>
       <c r="M55" t="n">
-        <v>0.68</v>
+        <v>0.675</v>
       </c>
       <c r="N55" t="n">
-        <v>-0</v>
+        <v>-0.005</v>
       </c>
       <c r="O55" t="n">
         <v>-0.74</v>
       </c>
       <c r="P55" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="Q55" t="n">
         <v>0.01</v>
@@ -3863,16 +3875,16 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.49</v>
+        <v>0.485</v>
       </c>
       <c r="E56" t="n">
-        <v>-0</v>
+        <v>-0.005</v>
       </c>
       <c r="F56" t="n">
         <v>-1.02</v>
       </c>
       <c r="G56" t="n">
-        <v>0.5</v>
+        <v>0.495</v>
       </c>
       <c r="H56" t="n">
         <v>0.01</v>
@@ -3881,7 +3893,7 @@
         <v>2.06</v>
       </c>
       <c r="J56" t="n">
-        <v>0.49</v>
+        <v>0.485</v>
       </c>
       <c r="K56" t="n">
         <v>-0.01</v>
@@ -3890,7 +3902,7 @@
         <v>-2.02</v>
       </c>
       <c r="M56" t="n">
-        <v>0.5</v>
+        <v>0.495</v>
       </c>
       <c r="N56" t="n">
         <v>0.01</v>
@@ -3902,7 +3914,7 @@
         <v>0.49</v>
       </c>
       <c r="Q56" t="n">
-        <v>-0</v>
+        <v>-0.005</v>
       </c>
       <c r="R56" t="n">
         <v>-1.01</v>
@@ -3987,16 +3999,16 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.08</v>
+        <v>0.079</v>
       </c>
       <c r="E58" t="n">
-        <v>-0</v>
+        <v>-0.001</v>
       </c>
       <c r="F58" t="n">
         <v>-1.25</v>
       </c>
       <c r="G58" t="n">
-        <v>0.08</v>
+        <v>0.079</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
@@ -4005,19 +4017,19 @@
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>0.08</v>
+        <v>0.081</v>
       </c>
       <c r="K58" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="L58" t="n">
         <v>2.53</v>
       </c>
       <c r="M58" t="n">
-        <v>0.08</v>
+        <v>0.079</v>
       </c>
       <c r="N58" t="n">
-        <v>-0</v>
+        <v>-0.002</v>
       </c>
       <c r="O58" t="n">
         <v>-2.47</v>
@@ -4026,7 +4038,7 @@
         <v>0.08</v>
       </c>
       <c r="Q58" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="R58" t="n">
         <v>1.27</v>

</xml_diff>